<commit_message>
feat: align CLI report generation with extension
- support manual work grouped under Nghiên cứu
- infer project paths from extension CSV exports
- sync Excel templates, formulas, and leave explanations
- support custom Excel filenames with safe characters
- add CLI and extension workbook parity tests
</commit_message>
<xml_diff>
--- a/src/kpi_report/templates/work_report.xlsx
+++ b/src/kpi_report/templates/work_report.xlsx
@@ -885,13 +885,6 @@
       <c r="I4" s="50" t="n"/>
       <c r="J4" s="50" t="n"/>
       <c r="K4" s="1" t="n"/>
-      <c r="L4" s="67" t="inlineStr">
-        <is>
-          <t>Thống Kê</t>
-        </is>
-      </c>
-      <c r="M4" s="68" t="n"/>
-      <c r="N4" s="1" t="n"/>
       <c r="O4" s="1" t="n"/>
       <c r="P4" s="1" t="n"/>
       <c r="Q4" s="1" t="n"/>
@@ -904,6 +897,13 @@
       <c r="X4" s="1" t="n"/>
       <c r="Y4" s="1" t="n"/>
       <c r="Z4" s="1" t="n"/>
+      <c r="L4" s="67" t="inlineStr">
+        <is>
+          <t>Thống Kê</t>
+        </is>
+      </c>
+      <c r="M4" s="68" t="n"/>
+      <c r="N4" s="1" t="n"/>
     </row>
     <row r="5" ht="15.75" customHeight="1" s="66">
       <c r="A5" s="1" t="n"/>
@@ -953,13 +953,6 @@
         </is>
       </c>
       <c r="K5" s="12" t="n"/>
-      <c r="L5" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng số task </t>
-        </is>
-      </c>
-      <c r="M5" s="25" t="n"/>
-      <c r="N5" s="1" t="n"/>
       <c r="O5" s="1" t="n"/>
       <c r="P5" s="1" t="n"/>
       <c r="Q5" s="1" t="n"/>
@@ -972,6 +965,13 @@
       <c r="X5" s="1" t="n"/>
       <c r="Y5" s="1" t="n"/>
       <c r="Z5" s="1" t="n"/>
+      <c r="L5" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng số task </t>
+        </is>
+      </c>
+      <c r="M5" s="25" t="n"/>
+      <c r="N5" s="1" t="n"/>
     </row>
     <row r="6" ht="15.75" customHeight="1" s="66">
       <c r="A6" s="1" t="n"/>
@@ -985,13 +985,6 @@
       <c r="I6" s="24" t="n"/>
       <c r="J6" s="24" t="n"/>
       <c r="K6" s="1" t="n"/>
-      <c r="L6" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng số task kế hoạch </t>
-        </is>
-      </c>
-      <c r="M6" s="25" t="n"/>
-      <c r="N6" s="1" t="n"/>
       <c r="O6" s="1" t="n"/>
       <c r="P6" s="1" t="n"/>
       <c r="Q6" s="1" t="n"/>
@@ -1004,17 +997,17 @@
       <c r="X6" s="1" t="n"/>
       <c r="Y6" s="1" t="n"/>
       <c r="Z6" s="1" t="n"/>
+      <c r="L6" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng số task kế hoạch </t>
+        </is>
+      </c>
+      <c r="M6" s="25" t="n"/>
+      <c r="N6" s="1" t="n"/>
     </row>
     <row r="7" ht="15.75" customHeight="1" s="66">
       <c r="A7" s="1" t="n"/>
       <c r="K7" s="1" t="n"/>
-      <c r="L7" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng số task phát sinh </t>
-        </is>
-      </c>
-      <c r="M7" s="25" t="n"/>
-      <c r="N7" s="1" t="n"/>
       <c r="O7" s="1" t="n"/>
       <c r="P7" s="1" t="n"/>
       <c r="Q7" s="1" t="n"/>
@@ -1027,23 +1020,17 @@
       <c r="X7" s="1" t="n"/>
       <c r="Y7" s="1" t="n"/>
       <c r="Z7" s="1" t="n"/>
+      <c r="L7" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng số task phát sinh </t>
+        </is>
+      </c>
+      <c r="M7" s="25" t="n"/>
+      <c r="N7" s="1" t="n"/>
     </row>
     <row r="8" ht="15.75" customHeight="1" s="66">
       <c r="A8" s="1" t="n"/>
       <c r="K8" s="1" t="n"/>
-      <c r="L8" s="25" t="inlineStr">
-        <is>
-          <t>Tổng thời gian làm việc theo lịch công ty (h)</t>
-        </is>
-      </c>
-      <c r="M8" s="25" t="n">
-        <v>192</v>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>Chỗ này luôn để là 192h</t>
-        </is>
-      </c>
       <c r="O8" s="1" t="n"/>
       <c r="P8" s="1" t="n"/>
       <c r="Q8" s="1" t="n"/>
@@ -1056,17 +1043,23 @@
       <c r="X8" s="1" t="n"/>
       <c r="Y8" s="1" t="n"/>
       <c r="Z8" s="1" t="n"/>
+      <c r="L8" s="25" t="inlineStr">
+        <is>
+          <t>Tổng thời gian làm việc theo lịch công ty (h)</t>
+        </is>
+      </c>
+      <c r="M8" s="25" t="n">
+        <v>192</v>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>Chỗ này luôn để là 192h</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15.75" customHeight="1" s="66">
       <c r="A9" s="1" t="n"/>
       <c r="K9" s="1" t="n"/>
-      <c r="L9" s="25" t="inlineStr">
-        <is>
-          <t>Tổng thời gian Estimate (h)</t>
-        </is>
-      </c>
-      <c r="M9" s="25" t="n"/>
-      <c r="N9" s="1" t="n"/>
       <c r="O9" s="1" t="n"/>
       <c r="P9" s="1" t="n"/>
       <c r="Q9" s="1" t="n"/>
@@ -1079,17 +1072,17 @@
       <c r="X9" s="1" t="n"/>
       <c r="Y9" s="1" t="n"/>
       <c r="Z9" s="1" t="n"/>
+      <c r="L9" s="25" t="inlineStr">
+        <is>
+          <t>Tổng thời gian Estimate (h)</t>
+        </is>
+      </c>
+      <c r="M9" s="25" t="n"/>
+      <c r="N9" s="1" t="n"/>
     </row>
     <row r="10" ht="15.75" customHeight="1" s="66">
       <c r="A10" s="1" t="n"/>
       <c r="K10" s="1" t="n"/>
-      <c r="L10" s="25" t="inlineStr">
-        <is>
-          <t>Tổng thời gian Spent time (h)</t>
-        </is>
-      </c>
-      <c r="M10" s="25" t="n"/>
-      <c r="N10" s="1" t="n"/>
       <c r="O10" s="1" t="n"/>
       <c r="P10" s="1" t="n"/>
       <c r="Q10" s="1" t="n"/>
@@ -1102,17 +1095,17 @@
       <c r="X10" s="1" t="n"/>
       <c r="Y10" s="1" t="n"/>
       <c r="Z10" s="1" t="n"/>
+      <c r="L10" s="25" t="inlineStr">
+        <is>
+          <t>Tổng thời gian Spent time (h)</t>
+        </is>
+      </c>
+      <c r="M10" s="25" t="n"/>
+      <c r="N10" s="1" t="n"/>
     </row>
     <row r="11" ht="15.75" customHeight="1" s="66">
       <c r="A11" s="1" t="n"/>
       <c r="K11" s="1" t="n"/>
-      <c r="L11" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng thời gian Spent time (h) của task kế hoạch </t>
-        </is>
-      </c>
-      <c r="M11" s="25" t="n"/>
-      <c r="N11" s="1" t="n"/>
       <c r="O11" s="1" t="n"/>
       <c r="P11" s="1" t="n"/>
       <c r="Q11" s="1" t="n"/>
@@ -1125,17 +1118,17 @@
       <c r="X11" s="1" t="n"/>
       <c r="Y11" s="1" t="n"/>
       <c r="Z11" s="1" t="n"/>
+      <c r="L11" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng thời gian Spent time (h) của task kế hoạch </t>
+        </is>
+      </c>
+      <c r="M11" s="25" t="n"/>
+      <c r="N11" s="1" t="n"/>
     </row>
     <row r="12" ht="15.75" customHeight="1" s="66">
       <c r="A12" s="1" t="n"/>
       <c r="K12" s="1" t="n"/>
-      <c r="L12" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng thời gian Spent time (h) của task phát sinh </t>
-        </is>
-      </c>
-      <c r="M12" s="25" t="n"/>
-      <c r="N12" s="1" t="n"/>
       <c r="O12" s="1" t="n"/>
       <c r="P12" s="1" t="n"/>
       <c r="Q12" s="1" t="n"/>
@@ -1148,17 +1141,17 @@
       <c r="X12" s="1" t="n"/>
       <c r="Y12" s="1" t="n"/>
       <c r="Z12" s="1" t="n"/>
+      <c r="L12" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng thời gian Spent time (h) của task phát sinh </t>
+        </is>
+      </c>
+      <c r="M12" s="25" t="n"/>
+      <c r="N12" s="1" t="n"/>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="66">
       <c r="A13" s="1" t="n"/>
       <c r="K13" s="1" t="n"/>
-      <c r="L13" s="13" t="inlineStr">
-        <is>
-          <t>Số lượng task chưa có Start date</t>
-        </is>
-      </c>
-      <c r="M13" s="25" t="n"/>
-      <c r="N13" s="1" t="n"/>
       <c r="O13" s="1" t="n"/>
       <c r="P13" s="1" t="n"/>
       <c r="Q13" s="1" t="n"/>
@@ -1171,17 +1164,17 @@
       <c r="X13" s="1" t="n"/>
       <c r="Y13" s="1" t="n"/>
       <c r="Z13" s="1" t="n"/>
+      <c r="L13" s="13" t="inlineStr">
+        <is>
+          <t>Số lượng task chưa có Start date</t>
+        </is>
+      </c>
+      <c r="M13" s="25" t="n"/>
+      <c r="N13" s="1" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="66">
       <c r="A14" s="1" t="n"/>
       <c r="K14" s="1" t="n"/>
-      <c r="L14" s="13" t="inlineStr">
-        <is>
-          <t>Số lượng task chưa có Due date</t>
-        </is>
-      </c>
-      <c r="M14" s="25" t="n"/>
-      <c r="N14" s="1" t="n"/>
       <c r="O14" s="1" t="n"/>
       <c r="P14" s="1" t="n"/>
       <c r="Q14" s="1" t="n"/>
@@ -1194,17 +1187,17 @@
       <c r="X14" s="1" t="n"/>
       <c r="Y14" s="1" t="n"/>
       <c r="Z14" s="1" t="n"/>
+      <c r="L14" s="13" t="inlineStr">
+        <is>
+          <t>Số lượng task chưa có Due date</t>
+        </is>
+      </c>
+      <c r="M14" s="25" t="n"/>
+      <c r="N14" s="1" t="n"/>
     </row>
     <row r="15" ht="15.75" customHeight="1" s="66">
       <c r="A15" s="1" t="n"/>
       <c r="K15" s="1" t="n"/>
-      <c r="L15" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Số lượng task chưa có Estimate </t>
-        </is>
-      </c>
-      <c r="M15" s="25" t="n"/>
-      <c r="N15" s="1" t="n"/>
       <c r="O15" s="1" t="n"/>
       <c r="P15" s="1" t="n"/>
       <c r="Q15" s="1" t="n"/>
@@ -1217,17 +1210,17 @@
       <c r="X15" s="1" t="n"/>
       <c r="Y15" s="1" t="n"/>
       <c r="Z15" s="1" t="n"/>
+      <c r="L15" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Số lượng task chưa có Estimate </t>
+        </is>
+      </c>
+      <c r="M15" s="25" t="n"/>
+      <c r="N15" s="1" t="n"/>
     </row>
     <row r="16" ht="15.75" customHeight="1" s="66">
       <c r="A16" s="1" t="n"/>
       <c r="K16" s="1" t="n"/>
-      <c r="L16" s="13" t="inlineStr">
-        <is>
-          <t>Số lượng task chưa có Spent time</t>
-        </is>
-      </c>
-      <c r="M16" s="25" t="n"/>
-      <c r="N16" s="1" t="n"/>
       <c r="O16" s="1" t="n"/>
       <c r="P16" s="1" t="n"/>
       <c r="Q16" s="1" t="n"/>
@@ -1240,17 +1233,17 @@
       <c r="X16" s="1" t="n"/>
       <c r="Y16" s="1" t="n"/>
       <c r="Z16" s="1" t="n"/>
+      <c r="L16" s="13" t="inlineStr">
+        <is>
+          <t>Số lượng task chưa có Spent time</t>
+        </is>
+      </c>
+      <c r="M16" s="25" t="n"/>
+      <c r="N16" s="1" t="n"/>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="66">
       <c r="A17" s="1" t="n"/>
       <c r="K17" s="1" t="n"/>
-      <c r="L17" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng số task đúng hạn </t>
-        </is>
-      </c>
-      <c r="M17" s="25" t="n"/>
-      <c r="N17" s="1" t="n"/>
       <c r="O17" s="1" t="n"/>
       <c r="P17" s="1" t="n"/>
       <c r="Q17" s="1" t="n"/>
@@ -1263,17 +1256,17 @@
       <c r="X17" s="1" t="n"/>
       <c r="Y17" s="1" t="n"/>
       <c r="Z17" s="1" t="n"/>
+      <c r="L17" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng số task đúng hạn </t>
+        </is>
+      </c>
+      <c r="M17" s="25" t="n"/>
+      <c r="N17" s="1" t="n"/>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="66">
       <c r="A18" s="1" t="n"/>
       <c r="K18" s="1" t="n"/>
-      <c r="L18" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng số task trễ hạn </t>
-        </is>
-      </c>
-      <c r="M18" s="25" t="n"/>
-      <c r="N18" s="1" t="n"/>
       <c r="O18" s="1" t="n"/>
       <c r="P18" s="1" t="n"/>
       <c r="Q18" s="1" t="n"/>
@@ -1286,13 +1279,17 @@
       <c r="X18" s="1" t="n"/>
       <c r="Y18" s="1" t="n"/>
       <c r="Z18" s="1" t="n"/>
+      <c r="L18" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng số task trễ hạn </t>
+        </is>
+      </c>
+      <c r="M18" s="25" t="n"/>
+      <c r="N18" s="1" t="n"/>
     </row>
     <row r="19" ht="15.75" customHeight="1" s="66">
       <c r="A19" s="1" t="n"/>
       <c r="K19" s="1" t="n"/>
-      <c r="L19" s="25" t="n"/>
-      <c r="M19" s="25" t="n"/>
-      <c r="N19" s="1" t="n"/>
       <c r="O19" s="1" t="n"/>
       <c r="P19" s="1" t="n"/>
       <c r="Q19" s="1" t="n"/>
@@ -1305,17 +1302,17 @@
       <c r="X19" s="1" t="n"/>
       <c r="Y19" s="1" t="n"/>
       <c r="Z19" s="1" t="n"/>
+      <c r="L19" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng số task không bị reopen </t>
+        </is>
+      </c>
+      <c r="M19" s="25" t="n"/>
+      <c r="N19" s="1" t="n"/>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="66">
       <c r="A20" s="1" t="n"/>
       <c r="K20" s="1" t="n"/>
-      <c r="L20" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng số task không bị reopen </t>
-        </is>
-      </c>
-      <c r="M20" s="25" t="n"/>
-      <c r="N20" s="1" t="n"/>
       <c r="O20" s="1" t="n"/>
       <c r="P20" s="1" t="n"/>
       <c r="Q20" s="1" t="n"/>
@@ -1328,17 +1325,17 @@
       <c r="X20" s="1" t="n"/>
       <c r="Y20" s="1" t="n"/>
       <c r="Z20" s="1" t="n"/>
+      <c r="L20" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng số task có bị reopen </t>
+        </is>
+      </c>
+      <c r="M20" s="25" t="n"/>
+      <c r="N20" s="1" t="n"/>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="66">
       <c r="A21" s="1" t="n"/>
       <c r="K21" s="1" t="n"/>
-      <c r="L21" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng số task có bị reopen </t>
-        </is>
-      </c>
-      <c r="M21" s="25" t="n"/>
-      <c r="N21" s="1" t="n"/>
       <c r="O21" s="1" t="n"/>
       <c r="P21" s="1" t="n"/>
       <c r="Q21" s="1" t="n"/>
@@ -1355,9 +1352,6 @@
     <row r="22" ht="15.75" customHeight="1" s="66">
       <c r="A22" s="1" t="n"/>
       <c r="K22" s="1" t="n"/>
-      <c r="L22" s="1" t="n"/>
-      <c r="M22" s="1" t="n"/>
-      <c r="N22" s="1" t="n"/>
       <c r="O22" s="1" t="n"/>
       <c r="P22" s="1" t="n"/>
       <c r="Q22" s="1" t="n"/>
@@ -1374,9 +1368,6 @@
     <row r="23" ht="15.75" customHeight="1" s="66">
       <c r="A23" s="1" t="n"/>
       <c r="K23" s="1" t="n"/>
-      <c r="L23" s="1" t="n"/>
-      <c r="M23" s="1" t="n"/>
-      <c r="N23" s="1" t="n"/>
       <c r="O23" s="1" t="n"/>
       <c r="P23" s="1" t="n"/>
       <c r="Q23" s="1" t="n"/>
@@ -1389,17 +1380,17 @@
       <c r="X23" s="1" t="n"/>
       <c r="Y23" s="1" t="n"/>
       <c r="Z23" s="1" t="n"/>
+      <c r="L23" s="67" t="inlineStr">
+        <is>
+          <t>Tỉ lệ (%)</t>
+        </is>
+      </c>
+      <c r="M23" s="68" t="n"/>
+      <c r="N23" s="1" t="n"/>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="66">
       <c r="A24" s="1" t="n"/>
       <c r="K24" s="1" t="n"/>
-      <c r="L24" s="67" t="inlineStr">
-        <is>
-          <t>Tỉ lệ (%)</t>
-        </is>
-      </c>
-      <c r="M24" s="68" t="n"/>
-      <c r="N24" s="1" t="n"/>
       <c r="O24" s="1" t="n"/>
       <c r="P24" s="1" t="n"/>
       <c r="Q24" s="1" t="n"/>
@@ -1412,20 +1403,20 @@
       <c r="X24" s="1" t="n"/>
       <c r="Y24" s="1" t="n"/>
       <c r="Z24" s="1" t="n"/>
+      <c r="L24" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Số lượng task chưa có Start date / Tổng số task </t>
+        </is>
+      </c>
+      <c r="M24" s="51">
+        <f>M13/M5*100</f>
+        <v/>
+      </c>
+      <c r="N24" s="1" t="n"/>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="66">
       <c r="A25" s="1" t="n"/>
       <c r="K25" s="1" t="n"/>
-      <c r="L25" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Số lượng task chưa có Start date / Tổng số task </t>
-        </is>
-      </c>
-      <c r="M25" s="51">
-        <f>M13/M5*100</f>
-        <v/>
-      </c>
-      <c r="N25" s="1" t="n"/>
       <c r="O25" s="1" t="n"/>
       <c r="P25" s="1" t="n"/>
       <c r="Q25" s="1" t="n"/>
@@ -1438,20 +1429,20 @@
       <c r="X25" s="1" t="n"/>
       <c r="Y25" s="1" t="n"/>
       <c r="Z25" s="1" t="n"/>
+      <c r="L25" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Số lượng task chưa có Due date / Tổng số task </t>
+        </is>
+      </c>
+      <c r="M25" s="51">
+        <f>M14/M5*100</f>
+        <v/>
+      </c>
+      <c r="N25" s="1" t="n"/>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="66">
       <c r="A26" s="1" t="n"/>
       <c r="K26" s="1" t="n"/>
-      <c r="L26" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Số lượng task chưa có Due date / Tổng số task </t>
-        </is>
-      </c>
-      <c r="M26" s="51">
-        <f>M14/M5*100</f>
-        <v/>
-      </c>
-      <c r="N26" s="1" t="n"/>
       <c r="O26" s="1" t="n"/>
       <c r="P26" s="1" t="n"/>
       <c r="Q26" s="1" t="n"/>
@@ -1464,20 +1455,20 @@
       <c r="X26" s="1" t="n"/>
       <c r="Y26" s="1" t="n"/>
       <c r="Z26" s="1" t="n"/>
+      <c r="L26" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Số lượng task chưa có Estimate / Tổng số task </t>
+        </is>
+      </c>
+      <c r="M26" s="51">
+        <f>M15/M5*100</f>
+        <v/>
+      </c>
+      <c r="N26" s="1" t="n"/>
     </row>
     <row r="27" ht="15.75" customHeight="1" s="66">
       <c r="A27" s="1" t="n"/>
       <c r="K27" s="1" t="n"/>
-      <c r="L27" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Số lượng task chưa có Estimate / Tổng số task </t>
-        </is>
-      </c>
-      <c r="M27" s="51">
-        <f>M15/M5*100</f>
-        <v/>
-      </c>
-      <c r="N27" s="1" t="n"/>
       <c r="O27" s="1" t="n"/>
       <c r="P27" s="1" t="n"/>
       <c r="Q27" s="1" t="n"/>
@@ -1490,20 +1481,20 @@
       <c r="X27" s="1" t="n"/>
       <c r="Y27" s="1" t="n"/>
       <c r="Z27" s="1" t="n"/>
+      <c r="L27" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Số lượng task chưa có Spent time / Tổng số task </t>
+        </is>
+      </c>
+      <c r="M27" s="51">
+        <f>M16/M5*100</f>
+        <v/>
+      </c>
+      <c r="N27" s="1" t="n"/>
     </row>
     <row r="28" ht="15.75" customHeight="1" s="66">
       <c r="A28" s="1" t="n"/>
       <c r="K28" s="1" t="n"/>
-      <c r="L28" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Số lượng task chưa có Spent time / Tổng số task </t>
-        </is>
-      </c>
-      <c r="M28" s="51">
-        <f>M16/M5*100</f>
-        <v/>
-      </c>
-      <c r="N28" s="1" t="n"/>
       <c r="O28" s="1" t="n"/>
       <c r="P28" s="1" t="n"/>
       <c r="Q28" s="1" t="n"/>
@@ -1516,20 +1507,20 @@
       <c r="X28" s="1" t="n"/>
       <c r="Y28" s="1" t="n"/>
       <c r="Z28" s="1" t="n"/>
+      <c r="L28" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng số task đúng hạn / Tổng số task </t>
+        </is>
+      </c>
+      <c r="M28" s="51">
+        <f>M17/M5*100</f>
+        <v/>
+      </c>
+      <c r="N28" s="1" t="n"/>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="66">
       <c r="A29" s="1" t="n"/>
       <c r="K29" s="1" t="n"/>
-      <c r="L29" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng số task đúng hạn / Tổng số task </t>
-        </is>
-      </c>
-      <c r="M29" s="51">
-        <f>M17/M5*100</f>
-        <v/>
-      </c>
-      <c r="N29" s="1" t="n"/>
       <c r="O29" s="1" t="n"/>
       <c r="P29" s="1" t="n"/>
       <c r="Q29" s="1" t="n"/>
@@ -1542,13 +1533,20 @@
       <c r="X29" s="1" t="n"/>
       <c r="Y29" s="1" t="n"/>
       <c r="Z29" s="1" t="n"/>
+      <c r="L29" s="25" t="inlineStr">
+        <is>
+          <t>Tổng số task trễ hạn / Tổng số task</t>
+        </is>
+      </c>
+      <c r="M29" s="51">
+        <f>M18/M5*100</f>
+        <v/>
+      </c>
+      <c r="N29" s="1" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n"/>
       <c r="K30" s="1" t="n"/>
-      <c r="L30" s="25" t="n"/>
-      <c r="M30" s="51" t="n"/>
-      <c r="N30" s="1" t="n"/>
       <c r="O30" s="1" t="n"/>
       <c r="P30" s="1" t="n"/>
       <c r="Q30" s="1" t="n"/>
@@ -1561,20 +1559,20 @@
       <c r="X30" s="1" t="n"/>
       <c r="Y30" s="1" t="n"/>
       <c r="Z30" s="1" t="n"/>
+      <c r="L30" s="25" t="inlineStr">
+        <is>
+          <t>Tổng số task không bị reopen / Tổng số task</t>
+        </is>
+      </c>
+      <c r="M30" s="51">
+        <f>M19/M5*100</f>
+        <v/>
+      </c>
+      <c r="N30" s="1" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n"/>
       <c r="K31" s="1" t="n"/>
-      <c r="L31" s="25" t="inlineStr">
-        <is>
-          <t>Tổng số task trễ hạn / Tổng số task</t>
-        </is>
-      </c>
-      <c r="M31" s="51">
-        <f>M18/M5*100</f>
-        <v/>
-      </c>
-      <c r="N31" s="1" t="n"/>
       <c r="O31" s="1" t="n"/>
       <c r="P31" s="1" t="n"/>
       <c r="Q31" s="1" t="n"/>
@@ -1587,20 +1585,20 @@
       <c r="X31" s="1" t="n"/>
       <c r="Y31" s="1" t="n"/>
       <c r="Z31" s="1" t="n"/>
+      <c r="L31" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng số task có bị reopen / Tổng số task </t>
+        </is>
+      </c>
+      <c r="M31" s="51">
+        <f>M20/M5*100</f>
+        <v/>
+      </c>
+      <c r="N31" s="1" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n"/>
       <c r="K32" s="1" t="n"/>
-      <c r="L32" s="25" t="inlineStr">
-        <is>
-          <t>Tổng số task không bị reopen / Tổng số task</t>
-        </is>
-      </c>
-      <c r="M32" s="51">
-        <f>M20/M5*100</f>
-        <v/>
-      </c>
-      <c r="N32" s="1" t="n"/>
       <c r="O32" s="1" t="n"/>
       <c r="P32" s="1" t="n"/>
       <c r="Q32" s="1" t="n"/>
@@ -1613,18 +1611,18 @@
       <c r="X32" s="1" t="n"/>
       <c r="Y32" s="1" t="n"/>
       <c r="Z32" s="1" t="n"/>
+      <c r="L32" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng số task phát sinh / Tổng số task </t>
+        </is>
+      </c>
+      <c r="M32" s="51">
+        <f>M7/M5*100</f>
+        <v/>
+      </c>
+      <c r="N32" s="1" t="n"/>
     </row>
     <row r="33" ht="15.75" customHeight="1" s="66">
-      <c r="L33" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng số task có bị reopen / Tổng số task </t>
-        </is>
-      </c>
-      <c r="M33" s="51">
-        <f>M21/M5*100</f>
-        <v/>
-      </c>
-      <c r="N33" s="1" t="n"/>
       <c r="O33" s="1" t="n"/>
       <c r="P33" s="1" t="n"/>
       <c r="Q33" s="1" t="n"/>
@@ -1637,18 +1635,18 @@
       <c r="X33" s="1" t="n"/>
       <c r="Y33" s="1" t="n"/>
       <c r="Z33" s="1" t="n"/>
+      <c r="L33" s="25" t="inlineStr">
+        <is>
+          <t>Tổng thời gian Spent time / Tổng thời gian làm việc theo lịch công ty</t>
+        </is>
+      </c>
+      <c r="M33" s="51">
+        <f>M10/M8*100</f>
+        <v/>
+      </c>
+      <c r="N33" s="1" t="n"/>
     </row>
     <row r="34" ht="15.75" customHeight="1" s="66">
-      <c r="L34" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng số task phát sinh / Tổng số task </t>
-        </is>
-      </c>
-      <c r="M34" s="51">
-        <f>M7/M5*100</f>
-        <v/>
-      </c>
-      <c r="N34" s="1" t="n"/>
       <c r="O34" s="1" t="n"/>
       <c r="P34" s="1" t="n"/>
       <c r="Q34" s="1" t="n"/>
@@ -1661,11 +1659,18 @@
       <c r="X34" s="1" t="n"/>
       <c r="Y34" s="1" t="n"/>
       <c r="Z34" s="1" t="n"/>
+      <c r="L34" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng thời gian Spent time / Tổng thời gian Estimate </t>
+        </is>
+      </c>
+      <c r="M34" s="51">
+        <f>M10/M9*100</f>
+        <v/>
+      </c>
+      <c r="N34" s="1" t="n"/>
     </row>
     <row r="35" ht="15.75" customHeight="1" s="66">
-      <c r="L35" s="25" t="n"/>
-      <c r="M35" s="51" t="n"/>
-      <c r="N35" s="1" t="n"/>
       <c r="O35" s="1" t="n"/>
       <c r="P35" s="1" t="n"/>
       <c r="Q35" s="1" t="n"/>
@@ -1678,18 +1683,18 @@
       <c r="X35" s="1" t="n"/>
       <c r="Y35" s="1" t="n"/>
       <c r="Z35" s="1" t="n"/>
+      <c r="L35" s="25" t="inlineStr">
+        <is>
+          <t>Tổng thời gian Spent time của task kế hoạch / Tổng thời gian Spent time</t>
+        </is>
+      </c>
+      <c r="M35" s="51">
+        <f>M11/M10*100</f>
+        <v/>
+      </c>
+      <c r="N35" s="1" t="n"/>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="66">
-      <c r="L36" s="25" t="inlineStr">
-        <is>
-          <t>Tổng thời gian Spent time / Tổng thời gian làm việc theo lịch công ty</t>
-        </is>
-      </c>
-      <c r="M36" s="51">
-        <f>M10/M8*100</f>
-        <v/>
-      </c>
-      <c r="N36" s="1" t="n"/>
       <c r="O36" s="1" t="n"/>
       <c r="P36" s="1" t="n"/>
       <c r="Q36" s="1" t="n"/>
@@ -1702,18 +1707,18 @@
       <c r="X36" s="1" t="n"/>
       <c r="Y36" s="1" t="n"/>
       <c r="Z36" s="1" t="n"/>
+      <c r="L36" s="25" t="inlineStr">
+        <is>
+          <t>Tổng thời gian Spent time của task phát sinh / Tổng thời gian Spent time</t>
+        </is>
+      </c>
+      <c r="M36" s="51">
+        <f>M12/M10*100</f>
+        <v/>
+      </c>
+      <c r="N36" s="1" t="n"/>
     </row>
     <row r="37">
-      <c r="L37" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng thời gian Spent time / Tổng thời gian Estimate </t>
-        </is>
-      </c>
-      <c r="M37" s="51">
-        <f>M10/M9*100</f>
-        <v/>
-      </c>
-      <c r="N37" s="1" t="n"/>
       <c r="O37" s="1" t="n"/>
       <c r="P37" s="1" t="n"/>
       <c r="Q37" s="1" t="n"/>
@@ -1728,16 +1733,6 @@
       <c r="Z37" s="1" t="n"/>
     </row>
     <row r="38" ht="15.75" customHeight="1" s="66">
-      <c r="L38" s="25" t="inlineStr">
-        <is>
-          <t>Tổng thời gian Spent time của task kế hoạch / Tổng thời gian Spent time</t>
-        </is>
-      </c>
-      <c r="M38" s="51">
-        <f>M11/M10*100</f>
-        <v/>
-      </c>
-      <c r="N38" s="1" t="n"/>
       <c r="O38" s="1" t="n"/>
       <c r="P38" s="1" t="n"/>
       <c r="Q38" s="1" t="n"/>
@@ -1752,16 +1747,6 @@
       <c r="Z38" s="1" t="n"/>
     </row>
     <row r="39" ht="15.75" customHeight="1" s="66">
-      <c r="L39" s="25" t="inlineStr">
-        <is>
-          <t>Tổng thời gian Spent time của task phát sinh / Tổng thời gian Spent time</t>
-        </is>
-      </c>
-      <c r="M39" s="51">
-        <f>M12/M10*100</f>
-        <v/>
-      </c>
-      <c r="N39" s="1" t="n"/>
       <c r="O39" s="1" t="n"/>
       <c r="P39" s="1" t="n"/>
       <c r="Q39" s="1" t="n"/>
@@ -2748,7 +2733,7 @@
     <row r="1010" ht="15.75" customHeight="1" s="66"/>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="L24:M24"/>
+    <mergeCell ref="L23:M23"/>
     <mergeCell ref="L4:M4"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
@@ -3074,7 +3059,7 @@
         <v>0.25</v>
       </c>
       <c r="F15" s="76">
-        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M27/100)</f>
+        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M26/100)</f>
         <v/>
       </c>
       <c r="G15" s="75">
@@ -3182,7 +3167,7 @@
         <v>0.25</v>
       </c>
       <c r="F20" s="76">
-        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M25/100)</f>
+        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M24/100)</f>
         <v/>
       </c>
       <c r="G20" s="75">
@@ -3290,7 +3275,7 @@
         <v>0.25</v>
       </c>
       <c r="F25" s="76">
-        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M26/100)</f>
+        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M25/100)</f>
         <v/>
       </c>
       <c r="G25" s="75">
@@ -3398,7 +3383,7 @@
         <v>0.25</v>
       </c>
       <c r="F30" s="76">
-        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M28/100)</f>
+        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M27/100)</f>
         <v/>
       </c>
       <c r="G30" s="75">
@@ -3510,7 +3495,7 @@
         <v>3</v>
       </c>
       <c r="F35" s="75">
-        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M36)</f>
+        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M33)</f>
         <v/>
       </c>
       <c r="G35" s="75">
@@ -3622,7 +3607,7 @@
         <v>3</v>
       </c>
       <c r="F40" s="83">
-        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M31/100)</f>
+        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M29/100)</f>
         <v/>
       </c>
       <c r="G40" s="81">
@@ -3730,7 +3715,7 @@
         <v>3</v>
       </c>
       <c r="F45" s="83">
-        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M33/100)</f>
+        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M31/100)</f>
         <v/>
       </c>
       <c r="G45" s="81">

</xml_diff>